<commit_message>
Tables with average per tool
</commit_message>
<xml_diff>
--- a/results/RQ3_data_per_tool/Outguess.xlsx
+++ b/results/RQ3_data_per_tool/Outguess.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study Materials\Year 3 (2022-2023)\Module 12\Resources\Experiment_code\Steganography-and-steganalysis-M12-resources\results\RQ3_data_per_tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9258A6E1-486A-46AE-8F73-D2470B500132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5EEDDD7-34D5-447C-AAC8-D0AAAD1C1080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Outguess" sheetId="1" r:id="rId1"/>

</xml_diff>